<commit_message>
CIMLR update commit 1
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/CIMLR/Supplement/Chisq_tests.xlsx
+++ b/Results/single_algorithm/CIMLR/Supplement/Chisq_tests.xlsx
@@ -29,10 +29,10 @@
     <t xml:space="preserve">Vital status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.832677982031382</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.366216575495905</t>
+    <t xml:space="preserve">0.968579407589046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00155157654444284</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -41,43 +41,43 @@
     <t xml:space="preserve">Ethnicity vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.244817080779635</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.81448791270295</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.036</t>
+    <t xml:space="preserve">0.169729629133553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.88532968096552</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.051</t>
   </si>
   <si>
     <t xml:space="preserve">Race vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.229316350127389</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.62076463375536</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.051</t>
+    <t xml:space="preserve">0.254213815690465</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.06800517266839</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.042</t>
   </si>
   <si>
     <t xml:space="preserve">Lymph node status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.722285745862054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.650668896987032</t>
+    <t xml:space="preserve">0.635222671233454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.225044742990889</t>
   </si>
   <si>
     <t xml:space="preserve">Histology vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.00061514493528327</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.3494672338262</t>
+    <t xml:space="preserve">0.000422339396976558</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.427374088555</t>
   </si>
   <si>
     <t xml:space="preserve">0.176</t>
@@ -86,67 +86,67 @@
     <t xml:space="preserve">Menopausal status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.362117148933096</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.33859487777134</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.023</t>
+    <t xml:space="preserve">0.243720998898003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.16962153607098</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.045</t>
   </si>
   <si>
     <t xml:space="preserve">PR status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.58691576020836e-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">39.1836715085833</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.241</t>
+    <t xml:space="preserve">3.11380736905481e-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39.1748392501928</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.252</t>
   </si>
   <si>
     <t xml:space="preserve">ER status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.49901116994509e-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.8214097745476</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.199</t>
+    <t xml:space="preserve">3.92064759596478e-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.7330028960813</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.21</t>
   </si>
   <si>
     <t xml:space="preserve">HER2 status vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.265043849142621</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.22433639914545</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.044</t>
+    <t xml:space="preserve">0.174074129248419</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.9690959334709</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.062</t>
   </si>
   <si>
     <t xml:space="preserve">Metastasis vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.423536841053528</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.71822955362334</t>
+    <t xml:space="preserve">0.999999999999998</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.50696541807422e-30</t>
   </si>
   <si>
     <t xml:space="preserve">Stage vs CIMLR cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.474207590842869</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.52420425664139</t>
+    <t xml:space="preserve">0.771774161189949</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.12196626161274</t>
   </si>
 </sst>
 </file>

</xml_diff>